<commit_message>
sms UI header verification testcases are added
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1707161580895841P6LSO</t>
+          <t>170716158089584XQCUMH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_1P6LSO</t>
+          <t>Template1_XQCUMH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1707161580898731P6LSO</t>
+          <t>170716158089873XQCUMH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_1P6LSO</t>
+          <t>Template2_XQCUMH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>827498174811P6LSO3</t>
+          <t>82749817481XQCUMH3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_1P6LSO</t>
+          <t>Template3_XQCUMH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>128498217981P6LSO4</t>
+          <t>12849821798XQCUMH4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_1P6LSO</t>
+          <t>Template4_XQCUMH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>812349821491P6LSO5</t>
+          <t>81234982149XQCUMH5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_1P6LSO</t>
+          <t>Template5_XQCUMH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>827498174811P6LSO6</t>
+          <t>82749817481XQCUMH6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_1P6LSO</t>
+          <t>Template6_XQCUMH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>128498217981P6LSO7</t>
+          <t>12849821798XQCUMH7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_1P6LSO</t>
+          <t>Template7_XQCUMH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>812349821491P6LSO8</t>
+          <t>81234982149XQCUMH8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_1P6LSO</t>
+          <t>Template8_XQCUMH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>827498174811P6LSO9</t>
+          <t>82749817481XQCUMH9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_1P6LSO</t>
+          <t>Template9_XQCUMH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>128498217981P6LSO10</t>
+          <t>12849821798XQCUMH10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_1P6LSO</t>
+          <t>Template10_XQCUMH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>812349821491P6LSO11</t>
+          <t>81234982149XQCUMH11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_1P6LSO</t>
+          <t>Template11_XQCUMH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
sms dlr, rcs headers verification
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584EOQ77H</t>
+          <t>170716158089584E811G2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_EOQ77H</t>
+          <t>Template1_E811G2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873EOQ77H</t>
+          <t>170716158089873E811G2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_EOQ77H</t>
+          <t>Template2_E811G2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>82749817481EOQ77H3</t>
+          <t>82749817481E811G23</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_EOQ77H</t>
+          <t>Template3_E811G2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798EOQ77H4</t>
+          <t>12849821798E811G24</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_EOQ77H</t>
+          <t>Template4_E811G2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81234982149EOQ77H5</t>
+          <t>81234982149E811G25</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_EOQ77H</t>
+          <t>Template5_E811G2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>82749817481EOQ77H6</t>
+          <t>82749817481E811G26</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_EOQ77H</t>
+          <t>Template6_E811G2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798EOQ77H7</t>
+          <t>12849821798E811G27</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_EOQ77H</t>
+          <t>Template7_E811G2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81234982149EOQ77H8</t>
+          <t>81234982149E811G28</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_EOQ77H</t>
+          <t>Template8_E811G2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82749817481EOQ77H9</t>
+          <t>82749817481E811G29</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_EOQ77H</t>
+          <t>Template9_E811G2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798EOQ77H10</t>
+          <t>12849821798E811G210</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_EOQ77H</t>
+          <t>Template10_E811G2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81234982149EOQ77H11</t>
+          <t>81234982149E811G211</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_EOQ77H</t>
+          <t>Template11_E811G2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
sms sender and template failed issue
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584640499</t>
+          <t>170716158089584495158</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_1Y12L7</t>
+          <t>Template1_T66JCH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873640499</t>
+          <t>170716158089873495158</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_1Y12L7</t>
+          <t>Template2_T66JCH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>827498174816404993</t>
+          <t>827498174814951583</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_1Y12L7</t>
+          <t>Template3_T66JCH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>128498217986404994</t>
+          <t>128498217984951584</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_1Y12L7</t>
+          <t>Template4_T66JCH</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>812349821496404995</t>
+          <t>812349821494951585</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_1Y12L7</t>
+          <t>Template5_T66JCH</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>827498174816404996</t>
+          <t>827498174814951586</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_1Y12L7</t>
+          <t>Template6_T66JCH</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>128498217986404997</t>
+          <t>128498217984951587</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_1Y12L7</t>
+          <t>Template7_T66JCH</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>812349821496404998</t>
+          <t>812349821494951588</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_1Y12L7</t>
+          <t>Template8_T66JCH</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>827498174816404999</t>
+          <t>827498174814951589</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_1Y12L7</t>
+          <t>Template9_T66JCH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1284982179864049910</t>
+          <t>1284982179849515810</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_1Y12L7</t>
+          <t>Template10_T66JCH</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>8123498214964049911</t>
+          <t>8123498214949515811</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_1Y12L7</t>
+          <t>Template11_T66JCH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>